<commit_message>
Add Shanghai-Suzhou-Wuzhen-Hangzhou itinerary (Mar 2027) from shanghai.xlsx
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -57,9 +57,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -447,6 +450,1332 @@
       <c r="C1" s="1" t="inlineStr">
         <is>
           <t>地点</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>03/08/2027</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>08:55</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>航班 吉隆坡 → 上海</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>03/08/2027</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>03/08/2027</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>03/08/2027</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>川沙公园</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>03/08/2027</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>川沙古镇</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>03/08/2027</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>静安寺</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>早餐 · 静安寺附近</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>宫宴 · 汉服妆造</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>陆家嘴</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>南京路步行街</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>外滩</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>城隍庙 · 豫园</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>03/10/2027</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>迪士尼小镇</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>03/10/2027</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>03/10/2027</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>上海迪士尼乐园</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>03/10/2027</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>迪士尼 · 跟拍（1 小时）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>03/10/2027</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>烟花 · 闭园</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>03/10/2027</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>03/11/2027</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>03/11/2027</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>上海站</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>03/11/2027</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>高铁 上海站 → 苏州站</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>03/11/2027</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>行乐酒店（苏州观前街平江路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>03/11/2027</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>午餐 · 酒店附近</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>03/11/2027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>虎丘风景区</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>03/11/2027</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>七里山塘千年古街</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>03/11/2027</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>03/12/2027</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>双塔市集</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>03/12/2027</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>行乐酒店（苏州观前街平江路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>03/12/2027</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>拙政园</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>03/12/2027</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>狮子林</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>03/12/2027</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>苏州恋爱博物馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>03/12/2027</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>平江路 · 午餐</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>03/12/2027</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>金鸡湖 · 东方之门</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>03/12/2027</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>早餐 · 酒店附近</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>行乐酒店（苏州观前街平江路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>苏州 → 乌镇</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>乌镇民宿</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>半城红妆汉服体验店</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>乌镇景区</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>回酒店 · 乌镇民宿</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>早茶客 · 桥里桥烧饼铺</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>乌镇民宿</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>乌镇 · 清晨漫步</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>午餐 · 退房</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>乌镇 → 杭州</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>钱王祠码头</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>三潭印月</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>曲院风荷</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>断桥残雪</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>武林夜市</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>早餐 · 酒店附近</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>上天竺法喜讲寺</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>灵隐寺</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>曲院风荷</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>太子湾公园</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>雷峰塔</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>杭州酒家（延安路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>早餐 · 酒店附近</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>大马弄 · 南宋街 · 河坊街</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>杭州东站</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>高铁 杭州东站 → 上海站</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>和颐至尊酒店（上海人民广场南京路步行街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>豫园 · 城隍庙</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>回酒店 · 和颐至尊酒店（上海人民广场南京路步行街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>03/17/2027</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>国际饭店西饼屋</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>03/17/2027</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>和颐至尊酒店（上海人民广场南京路步行街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>03/17/2027</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>03/17/2027</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>16:05</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>航班 上海 → 吉隆坡</t>
         </is>
       </c>
     </row>
@@ -461,7 +1790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -477,6 +1806,714 @@
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>地点</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>03/08/2027</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>新川饮食</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>03/08/2027</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>老味茶屋</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>03/08/2027</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>老毛烧饼</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>03/08/2027</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>上海老式葱油饼</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>03/08/2027</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>忘不了酸菜鱼</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>03/08/2027</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>老街人家农家菜</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>03/08/2027</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>老街菜饭</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>百丘（PAIN CHAUD）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>鼎福记小笼馄饨</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>莱莱小笼（乔艾静安店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>德兴馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>鲜得来排骨年糕（山西南路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>泸西老弄堂面馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>沈大成</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>莱莱小笼包（南京东路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>大壶春（四川中路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>03/10/2027</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>猪手饭（皮诺丘乡村厨房）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>03/10/2027</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>新旺茶餐室（迪士尼小镇）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>03/10/2027</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>酸萝卜鸭腿（漫月出口餐车）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>03/11/2027</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>万福兴（凤凰街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>03/11/2027</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>鑫震源 · 苏式大虾生煎</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>03/11/2027</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>哑巴生煎（海市山塘 45 号）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>03/11/2027</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>秋娟小吃店</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>03/11/2027</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>沈万三 · 江南卤味（山塘街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>03/12/2027</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>老客满蛋</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>03/12/2027</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>大孃孃苏式糖水（双塔市集店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>03/12/2027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>江南米造局（双塔市集店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>03/12/2027</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>苏拾里</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>03/12/2027</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>苏外婆</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>万福兴（凤凰街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>鑫震源 · 苏式大虾生煎</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>滋啦啦油煎铺</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>吴妈馄饨</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>锦记糕点铺</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>书生羊肉面</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>乌镇酱鸭店</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>永平粉团铺</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>锦岸私房菜</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>桥里桥烧饼铺</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>知味观</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>杭州绿豆糕（河坊街）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>富春王记烧饼（中山中路店总店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>红帽叔叔包子</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>潘老板炸鸡腿</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>熨斗大姐 葱包烩儿</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>新疆烤包子</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>李喜欢虾滑</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>龙井茉莉花豆浆</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>游埠豆浆（河坊街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>王氏烧饼无矾油条</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>杭州酒家（延安路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>游埠豆浆（河坊街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>王氏烧饼无矾油条</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>外婆家（南京东路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>光明邨大酒家</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>小杨生煎（人民广场店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>03/17/2027</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>国际饭店西饼屋</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Return flight MH389 15:25
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -1770,12 +1770,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>航班 上海 → 吉隆坡</t>
+          <t>航班 MH389 上海 → 吉隆坡</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fly out 3/16: skip Shanghai night, direct to PVG for MH389
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>07:45</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>杭州东站</t>
+          <t>杭州 → 浦东机场</t>
         </is>
       </c>
     </row>
@@ -1651,129 +1651,10 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
-        <is>
-          <t>高铁 杭州东站 → 上海站</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>14:30</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>和颐至尊酒店（上海人民广场南京路步行街店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>豫园 · 城隍庙</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>21:00</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>回酒店 · 和颐至尊酒店（上海人民广场南京路步行街店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>03/17/2027</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>国际饭店西饼屋</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>03/17/2027</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>和颐至尊酒店（上海人民广场南京路步行街店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>03/17/2027</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>上海浦东国际机场</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>03/17/2027</t>
-        </is>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>15:25</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>
@@ -1790,7 +1671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:B56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2466,54 +2347,6 @@
       <c r="B56" t="inlineStr">
         <is>
           <t>王氏烧饼无矾油条</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>外婆家（南京东路店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>光明邨大酒家</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>小杨生煎（人民广场店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>03/17/2027</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>国际饭店西饼屋</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day 9: public transport to PVG
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>07:45</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>杭州 → 浦东机场</t>
+          <t>杭州东站</t>
         </is>
       </c>
     </row>
@@ -1651,10 +1651,61 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>上海南站</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>景洪路站</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
           <t>15:25</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>

</xml_diff>

<commit_message>
Day 5: add 月光码头 before 金鸡湖
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1056,12 +1056,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>金鸡湖 · 东方之门</t>
+          <t>月光码头</t>
         </is>
       </c>
     </row>
@@ -1073,29 +1073,29 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
+          <t>金鸡湖 · 东方之门</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1124,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>苏州 → 乌镇</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1141,12 +1141,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>苏州 → 乌镇</t>
         </is>
       </c>
     </row>
@@ -1158,12 +1158,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>半城红妆汉服体验店</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1175,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>乌镇景区</t>
+          <t>半城红妆汉服体验店</t>
         </is>
       </c>
     </row>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>回酒店 · 乌镇民宿</t>
+          <t>乌镇景区</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>早茶客 · 桥里桥烧饼铺</t>
+          <t>回酒店 · 乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>早茶客 · 桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -1243,12 +1243,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>乌镇 · 清晨漫步</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1260,12 +1260,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>午餐 · 退房</t>
+          <t>乌镇 · 清晨漫步</t>
         </is>
       </c>
     </row>
@@ -1277,12 +1277,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>乌镇 → 杭州</t>
+          <t>午餐 · 退房</t>
         </is>
       </c>
     </row>
@@ -1294,12 +1294,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>乌镇 → 杭州</t>
         </is>
       </c>
     </row>
@@ -1311,12 +1311,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>钱王祠码头</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1328,12 +1328,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>三潭印月</t>
+          <t>钱王祠码头</t>
         </is>
       </c>
     </row>
@@ -1345,12 +1345,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>三潭印月</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>断桥残雪</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>武林夜市</t>
+          <t>断桥残雪</t>
         </is>
       </c>
     </row>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>武林夜市</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1435,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1447,12 +1447,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>上天竺法喜讲寺</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1464,12 +1464,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>灵隐寺</t>
+          <t>上天竺法喜讲寺</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>灵隐寺</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>太子湾公园</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>雷峰塔</t>
+          <t>太子湾公园</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>雷峰塔</t>
         </is>
       </c>
     </row>
@@ -1549,29 +1549,29 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>03/16/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1600,12 +1600,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>大马弄 · 南宋街 · 河坊街</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1617,12 +1617,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>大马弄 · 南宋街 · 河坊街</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>杭州东站</t>
+          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1651,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>上海南站</t>
+          <t>杭州东站</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>景洪路站</t>
+          <t>上海南站</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>上海浦东国际机场</t>
+          <t>景洪路站</t>
         </is>
       </c>
     </row>
@@ -1702,10 +1702,27 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
           <t>15:25</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>

</xml_diff>

<commit_message>
Day 8: walk 苏堤 after 曲院风荷
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>太子湾公园</t>
+          <t>苏堤</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>雷峰塔</t>
+          <t>太子湾公园</t>
         </is>
       </c>
     </row>
@@ -1549,12 +1549,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>雷峰塔</t>
         </is>
       </c>
     </row>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>03/16/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1605,7 +1605,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1617,12 +1617,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>大马弄 · 南宋街 · 河坊街</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>大马弄 · 南宋街 · 河坊街</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1651,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>杭州东站</t>
+          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>上海南站</t>
+          <t>杭州东站</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>景洪路站</t>
+          <t>上海南站</t>
         </is>
       </c>
     </row>
@@ -1702,12 +1702,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>上海浦东国际机场</t>
+          <t>景洪路站</t>
         </is>
       </c>
     </row>
@@ -1719,10 +1719,27 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
           <t>15:25</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>

</xml_diff>

<commit_message>
Day 8: 湖滨银泰in77 after dinner
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1583,29 +1583,29 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>湖滨银泰 in77</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>03/16/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>大马弄 · 南宋街 · 河坊街</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1651,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>大马弄 · 南宋街 · 河坊街</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>杭州东站</t>
+          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>上海南站</t>
+          <t>杭州东站</t>
         </is>
       </c>
     </row>
@@ -1702,12 +1702,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>景洪路站</t>
+          <t>上海南站</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>上海浦东国际机场</t>
+          <t>景洪路站</t>
         </is>
       </c>
     </row>
@@ -1736,10 +1736,27 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
           <t>15:25</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>

</xml_diff>

<commit_message>
Day 5: start later
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -954,7 +954,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">

</xml_diff>

<commit_message>
Day 1: dinner at 国营工农饭店
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -546,29 +546,29 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>晚餐 · 国营工农饭店</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>03/09/2027</t>
+          <t>03/08/2027</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>静安寺</t>
+          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>静安寺</t>
         </is>
       </c>
     </row>
@@ -597,12 +597,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>早餐 · 静安寺附近</t>
+          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>宫宴 · 汉服妆造</t>
+          <t>早餐 · 静安寺附近</t>
         </is>
       </c>
     </row>
@@ -631,12 +631,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>陆家嘴</t>
+          <t>宫宴 · 汉服妆造</t>
         </is>
       </c>
     </row>
@@ -648,12 +648,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>南京路步行街</t>
+          <t>陆家嘴</t>
         </is>
       </c>
     </row>
@@ -665,12 +665,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>外滩</t>
+          <t>南京路步行街</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>城隍庙 · 豫园</t>
+          <t>外滩</t>
         </is>
       </c>
     </row>
@@ -699,29 +699,29 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>城隍庙 · 豫园</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/09/2027</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>迪士尼小镇</t>
+          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>迪士尼小镇</t>
         </is>
       </c>
     </row>
@@ -750,12 +750,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>上海迪士尼乐园</t>
+          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -767,12 +767,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>迪士尼 · 跟拍（1 小时）</t>
+          <t>上海迪士尼乐园</t>
         </is>
       </c>
     </row>
@@ -784,12 +784,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>烟花 · 闭园</t>
+          <t>迪士尼 · 跟拍（1 小时）</t>
         </is>
       </c>
     </row>
@@ -801,29 +801,29 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>烟花 · 闭园</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -835,12 +835,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>上海站</t>
+          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -852,12 +852,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>高铁 上海站 → 苏州站</t>
+          <t>上海站</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>高铁 上海站 → 苏州站</t>
         </is>
       </c>
     </row>
@@ -886,12 +886,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>午餐 · 酒店附近</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -903,12 +903,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>虎丘风景区</t>
+          <t>午餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -920,12 +920,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>七里山塘千年古街</t>
+          <t>虎丘风景区</t>
         </is>
       </c>
     </row>
@@ -937,29 +937,29 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
+          <t>七里山塘千年古街</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>双塔市集</t>
+          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>双塔市集</t>
         </is>
       </c>
     </row>
@@ -988,12 +988,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>拙政园</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1005,12 +1005,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>狮子林</t>
+          <t>拙政园</t>
         </is>
       </c>
     </row>
@@ -1022,12 +1022,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>平江路</t>
+          <t>狮子林</t>
         </is>
       </c>
     </row>
@@ -1039,12 +1039,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>午餐 · 平江路</t>
+          <t>平江路</t>
         </is>
       </c>
     </row>
@@ -1056,12 +1056,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>月光码头</t>
+          <t>午餐 · 平江路</t>
         </is>
       </c>
     </row>
@@ -1073,12 +1073,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>金鸡湖 · 东方之门</t>
+          <t>月光码头</t>
         </is>
       </c>
     </row>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
+          <t>金鸡湖 · 东方之门</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1141,12 +1141,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>苏州 → 乌镇</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1158,12 +1158,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>苏州 → 乌镇</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1175,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>半城红妆汉服体验店</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1192,12 +1192,12 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>乌镇景区</t>
+          <t>半城红妆汉服体验店</t>
         </is>
       </c>
     </row>
@@ -1209,29 +1209,29 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>回酒店 · 乌镇民宿</t>
+          <t>乌镇景区</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>早茶客 · 桥里桥烧饼铺</t>
+          <t>回酒店 · 乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>早茶客 · 桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -1260,12 +1260,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>乌镇 · 清晨漫步</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1277,12 +1277,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>午餐 · 退房</t>
+          <t>乌镇 · 清晨漫步</t>
         </is>
       </c>
     </row>
@@ -1294,12 +1294,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>乌镇 → 杭州</t>
+          <t>午餐 · 退房</t>
         </is>
       </c>
     </row>
@@ -1311,12 +1311,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>乌镇 → 杭州</t>
         </is>
       </c>
     </row>
@@ -1328,12 +1328,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>钱王祠码头</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1345,12 +1345,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>三潭印月</t>
+          <t>钱王祠码头</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>三潭印月</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>断桥残雪</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1396,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>武林夜市</t>
+          <t>断桥残雪</t>
         </is>
       </c>
     </row>
@@ -1413,29 +1413,29 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>武林夜市</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1452,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1464,12 +1464,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>上天竺法喜讲寺</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>灵隐寺</t>
+          <t>上天竺法喜讲寺</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>灵隐寺</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>苏堤</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>太子湾公园</t>
+          <t>苏堤</t>
         </is>
       </c>
     </row>
@@ -1549,12 +1549,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>雷峰塔</t>
+          <t>太子湾公园</t>
         </is>
       </c>
     </row>
@@ -1566,12 +1566,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>雷峰塔</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1583,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>湖滨银泰 in77</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>湖滨银泰 in77</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>03/16/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1651,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>大马弄 · 南宋街 · 河坊街</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>大马弄 · 南宋街 · 河坊街</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>杭州东站</t>
+          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1702,12 +1702,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>上海南站</t>
+          <t>杭州东站</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>景洪路站</t>
+          <t>上海南站</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>上海浦东国际机场</t>
+          <t>景洪路站</t>
         </is>
       </c>
     </row>
@@ -1753,10 +1753,27 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
           <t>15:25</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>
@@ -1773,7 +1790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1860,19 +1877,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>老街人家农家菜</t>
+          <t>国营工农饭店</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>03/08/2027</t>
+          <t>03/09/2027</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>老街菜饭</t>
+          <t>百丘（PAIN CHAUD）</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1901,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>百丘（PAIN CHAUD）</t>
+          <t>鼎福记小笼馄饨</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1913,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>鼎福记小笼馄饨</t>
+          <t>莱莱小笼（乔艾静安店）</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1925,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>莱莱小笼（乔艾静安店）</t>
+          <t>德兴馆</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1937,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>德兴馆</t>
+          <t>鲜得来排骨年糕（山西南路店）</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1949,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>鲜得来排骨年糕（山西南路店）</t>
+          <t>泸西老弄堂面馆</t>
         </is>
       </c>
     </row>
@@ -1944,7 +1961,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>泸西老弄堂面馆</t>
+          <t>沈大成</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1973,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>沈大成</t>
+          <t>莱莱小笼包（南京东路店）</t>
         </is>
       </c>
     </row>
@@ -1968,19 +1985,19 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>莱莱小笼包（南京东路店）</t>
+          <t>大壶春（四川中路店）</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>03/09/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>大壶春（四川中路店）</t>
+          <t>猪手饭（皮诺丘乡村厨房）</t>
         </is>
       </c>
     </row>
@@ -1992,7 +2009,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>猪手饭（皮诺丘乡村厨房）</t>
+          <t>新旺茶餐室（迪士尼小镇）</t>
         </is>
       </c>
     </row>
@@ -2004,19 +2021,19 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>新旺茶餐室（迪士尼小镇）</t>
+          <t>酸萝卜鸭腿（漫月出口餐车）</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>酸萝卜鸭腿（漫月出口餐车）</t>
+          <t>万福兴（凤凰街店）</t>
         </is>
       </c>
     </row>
@@ -2028,7 +2045,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>万福兴（凤凰街店）</t>
+          <t>鑫震源 · 苏式大虾生煎</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2057,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>鑫震源 · 苏式大虾生煎</t>
+          <t>哑巴生煎（海市山塘 45 号）</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2069,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>哑巴生煎（海市山塘 45 号）</t>
+          <t>秋娟小吃店</t>
         </is>
       </c>
     </row>
@@ -2064,19 +2081,19 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>秋娟小吃店</t>
+          <t>沈万三 · 江南卤味（山塘街店）</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>沈万三 · 江南卤味（山塘街店）</t>
+          <t>老客满蛋</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2105,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>老客满蛋</t>
+          <t>大孃孃苏式糖水（双塔市集店）</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2117,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>大孃孃苏式糖水（双塔市集店）</t>
+          <t>江南米造局（双塔市集店）</t>
         </is>
       </c>
     </row>
@@ -2112,7 +2129,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>江南米造局（双塔市集店）</t>
+          <t>苏拾里</t>
         </is>
       </c>
     </row>
@@ -2124,19 +2141,19 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>苏拾里</t>
+          <t>苏外婆</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>苏外婆</t>
+          <t>万福兴（凤凰街店）</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2165,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>万福兴（凤凰街店）</t>
+          <t>鑫震源 · 苏式大虾生煎</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2177,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>鑫震源 · 苏式大虾生煎</t>
+          <t>滋啦啦油煎铺</t>
         </is>
       </c>
     </row>
@@ -2172,7 +2189,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>滋啦啦油煎铺</t>
+          <t>吴妈馄饨</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2201,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>吴妈馄饨</t>
+          <t>锦记糕点铺</t>
         </is>
       </c>
     </row>
@@ -2196,7 +2213,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>锦记糕点铺</t>
+          <t>书生羊肉面</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2225,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>书生羊肉面</t>
+          <t>乌镇酱鸭店</t>
         </is>
       </c>
     </row>
@@ -2220,7 +2237,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>乌镇酱鸭店</t>
+          <t>永平粉团铺</t>
         </is>
       </c>
     </row>
@@ -2232,19 +2249,19 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>永平粉团铺</t>
+          <t>锦岸私房菜</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>锦岸私房菜</t>
+          <t>桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -2256,7 +2273,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>桥里桥烧饼铺</t>
+          <t>知味观</t>
         </is>
       </c>
     </row>
@@ -2268,7 +2285,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>知味观</t>
+          <t>杭州绿豆糕（河坊街）</t>
         </is>
       </c>
     </row>
@@ -2280,7 +2297,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>杭州绿豆糕（河坊街）</t>
+          <t>富春王记烧饼（中山中路店总店）</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2309,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>富春王记烧饼（中山中路店总店）</t>
+          <t>红帽叔叔包子</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2321,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>红帽叔叔包子</t>
+          <t>潘老板炸鸡腿</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2333,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>潘老板炸鸡腿</t>
+          <t>熨斗大姐 葱包烩儿</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2345,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>熨斗大姐 葱包烩儿</t>
+          <t>新疆烤包子</t>
         </is>
       </c>
     </row>
@@ -2340,7 +2357,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>新疆烤包子</t>
+          <t>李喜欢虾滑</t>
         </is>
       </c>
     </row>
@@ -2352,19 +2369,19 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>李喜欢虾滑</t>
+          <t>龙井茉莉花豆浆</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>龙井茉莉花豆浆</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2393,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -2388,7 +2405,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
+          <t>王氏烧饼无矾油条</t>
         </is>
       </c>
     </row>
@@ -2400,19 +2417,19 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>王氏烧饼无矾油条</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/16/2027</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2441,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -2435,18 +2452,6 @@
         </is>
       </c>
       <c r="B55" t="inlineStr">
-        <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
         <is>
           <t>王氏烧饼无矾油条</t>
         </is>

</xml_diff>

<commit_message>
Day 2: hotel -> 川沙站 -> 静安寺
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -585,7 +585,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>静安寺</t>
+          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -597,12 +597,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>川沙地铁站</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>早餐 · 静安寺附近</t>
+          <t>静安寺</t>
         </is>
       </c>
     </row>
@@ -631,12 +631,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>宫宴 · 汉服妆造</t>
+          <t>早餐 · 静安寺附近</t>
         </is>
       </c>
     </row>
@@ -648,12 +648,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>陆家嘴</t>
+          <t>宫宴 · 汉服妆造</t>
         </is>
       </c>
     </row>
@@ -665,12 +665,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>南京路步行街</t>
+          <t>陆家嘴</t>
         </is>
       </c>
     </row>
@@ -682,12 +682,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>外滩</t>
+          <t>南京路步行街</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>城隍庙 · 豫园</t>
+          <t>外滩</t>
         </is>
       </c>
     </row>
@@ -716,29 +716,29 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>城隍庙 · 豫园</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/09/2027</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>迪士尼小镇</t>
+          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>迪士尼小镇</t>
         </is>
       </c>
     </row>
@@ -767,12 +767,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>上海迪士尼乐园</t>
+          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -784,12 +784,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>迪士尼 · 跟拍（1 小时）</t>
+          <t>上海迪士尼乐园</t>
         </is>
       </c>
     </row>
@@ -801,12 +801,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>烟花 · 闭园</t>
+          <t>迪士尼 · 跟拍（1 小时）</t>
         </is>
       </c>
     </row>
@@ -818,29 +818,29 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>烟花 · 闭园</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -852,12 +852,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>上海站</t>
+          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>高铁 上海站 → 苏州站</t>
+          <t>上海站</t>
         </is>
       </c>
     </row>
@@ -886,12 +886,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>高铁 上海站 → 苏州站</t>
         </is>
       </c>
     </row>
@@ -903,12 +903,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>午餐 · 酒店附近</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -920,12 +920,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>虎丘风景区</t>
+          <t>午餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -937,12 +937,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>七里山塘千年古街</t>
+          <t>虎丘风景区</t>
         </is>
       </c>
     </row>
@@ -954,29 +954,29 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
+          <t>七里山塘千年古街</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>双塔市集</t>
+          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>双塔市集</t>
         </is>
       </c>
     </row>
@@ -1005,12 +1005,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>拙政园</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1022,12 +1022,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>狮子林</t>
+          <t>拙政园</t>
         </is>
       </c>
     </row>
@@ -1039,12 +1039,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>平江路</t>
+          <t>狮子林</t>
         </is>
       </c>
     </row>
@@ -1056,12 +1056,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>午餐 · 平江路</t>
+          <t>平江路</t>
         </is>
       </c>
     </row>
@@ -1073,12 +1073,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>月光码头</t>
+          <t>午餐 · 平江路</t>
         </is>
       </c>
     </row>
@@ -1090,12 +1090,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>金鸡湖 · 东方之门</t>
+          <t>月光码头</t>
         </is>
       </c>
     </row>
@@ -1107,29 +1107,29 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
+          <t>金鸡湖 · 东方之门</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1158,12 +1158,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>苏州 → 乌镇</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1175,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>苏州 → 乌镇</t>
         </is>
       </c>
     </row>
@@ -1192,12 +1192,12 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>半城红妆汉服体验店</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1209,12 +1209,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>乌镇景区</t>
+          <t>半城红妆汉服体验店</t>
         </is>
       </c>
     </row>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>回酒店 · 乌镇民宿</t>
+          <t>乌镇景区</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>早茶客 · 桥里桥烧饼铺</t>
+          <t>回酒店 · 乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>早茶客 · 桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -1277,12 +1277,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>乌镇 · 清晨漫步</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1294,12 +1294,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>午餐 · 退房</t>
+          <t>乌镇 · 清晨漫步</t>
         </is>
       </c>
     </row>
@@ -1311,12 +1311,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>乌镇 → 杭州</t>
+          <t>午餐 · 退房</t>
         </is>
       </c>
     </row>
@@ -1328,12 +1328,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>乌镇 → 杭州</t>
         </is>
       </c>
     </row>
@@ -1345,12 +1345,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>钱王祠码头</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>三潭印月</t>
+          <t>钱王祠码头</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>三潭印月</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1396,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>断桥残雪</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1413,12 +1413,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>武林夜市</t>
+          <t>断桥残雪</t>
         </is>
       </c>
     </row>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>武林夜市</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1469,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>上天竺法喜讲寺</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>灵隐寺</t>
+          <t>上天竺法喜讲寺</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>灵隐寺</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>苏堤</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1549,12 +1549,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>太子湾公园</t>
+          <t>苏堤</t>
         </is>
       </c>
     </row>
@@ -1566,12 +1566,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>雷峰塔</t>
+          <t>太子湾公园</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1583,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>雷峰塔</t>
         </is>
       </c>
     </row>
@@ -1600,12 +1600,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>湖滨银泰 in77</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
@@ -1617,29 +1617,29 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>湖滨银泰 in77</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>03/16/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>大马弄 · 南宋街 · 河坊街</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>大马弄 · 南宋街 · 河坊街</t>
         </is>
       </c>
     </row>
@@ -1702,12 +1702,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>杭州东站</t>
+          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>上海南站</t>
+          <t>杭州东站</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>景洪路站</t>
+          <t>上海南站</t>
         </is>
       </c>
     </row>
@@ -1753,12 +1753,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>上海浦东国际机场</t>
+          <t>景洪路站</t>
         </is>
       </c>
     </row>
@@ -1770,10 +1770,27 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
           <t>15:25</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C80" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>

</xml_diff>

<commit_message>
Day 2: breakfast at 莱莱小笼
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -631,12 +631,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>早餐 · 静安寺附近</t>
+          <t>早餐 · 莱莱小笼（乔艾静安店）</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B55"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1906,7 +1906,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>百丘（PAIN CHAUD）</t>
+          <t>莱莱小笼（乔艾静安店）</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>鼎福记小笼馄饨</t>
+          <t>德兴馆</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1930,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>莱莱小笼（乔艾静安店）</t>
+          <t>鲜得来排骨年糕（山西南路店）</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>德兴馆</t>
+          <t>泸西老弄堂面馆</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>鲜得来排骨年糕（山西南路店）</t>
+          <t>沈大成</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>泸西老弄堂面馆</t>
+          <t>莱莱小笼包（南京东路店）</t>
         </is>
       </c>
     </row>
@@ -1978,31 +1978,31 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>沈大成</t>
+          <t>大壶春（四川中路店）</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>03/09/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>莱莱小笼包（南京东路店）</t>
+          <t>猪手饭（皮诺丘乡村厨房）</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>03/09/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>大壶春（四川中路店）</t>
+          <t>新旺茶餐室（迪士尼小镇）</t>
         </is>
       </c>
     </row>
@@ -2014,31 +2014,31 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>猪手饭（皮诺丘乡村厨房）</t>
+          <t>酸萝卜鸭腿（漫月出口餐车）</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>新旺茶餐室（迪士尼小镇）</t>
+          <t>万福兴（凤凰街店）</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>酸萝卜鸭腿（漫月出口餐车）</t>
+          <t>鑫震源 · 苏式大虾生煎</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2050,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>万福兴（凤凰街店）</t>
+          <t>哑巴生煎（海市山塘 45 号）</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>鑫震源 · 苏式大虾生煎</t>
+          <t>秋娟小吃店</t>
         </is>
       </c>
     </row>
@@ -2074,31 +2074,31 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>哑巴生煎（海市山塘 45 号）</t>
+          <t>沈万三 · 江南卤味（山塘街店）</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>秋娟小吃店</t>
+          <t>老客满蛋</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>沈万三 · 江南卤味（山塘街店）</t>
+          <t>大孃孃苏式糖水（双塔市集店）</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2110,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>老客满蛋</t>
+          <t>江南米造局（双塔市集店）</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2122,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>大孃孃苏式糖水（双塔市集店）</t>
+          <t>苏拾里</t>
         </is>
       </c>
     </row>
@@ -2134,31 +2134,31 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>江南米造局（双塔市集店）</t>
+          <t>苏外婆</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>苏拾里</t>
+          <t>万福兴（凤凰街店）</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>苏外婆</t>
+          <t>鑫震源 · 苏式大虾生煎</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2170,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>万福兴（凤凰街店）</t>
+          <t>滋啦啦油煎铺</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>鑫震源 · 苏式大虾生煎</t>
+          <t>吴妈馄饨</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>滋啦啦油煎铺</t>
+          <t>锦记糕点铺</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>吴妈馄饨</t>
+          <t>书生羊肉面</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>锦记糕点铺</t>
+          <t>乌镇酱鸭店</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>书生羊肉面</t>
+          <t>永平粉团铺</t>
         </is>
       </c>
     </row>
@@ -2242,31 +2242,31 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>乌镇酱鸭店</t>
+          <t>锦岸私房菜</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>永平粉团铺</t>
+          <t>桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>锦岸私房菜</t>
+          <t>知味观</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>桥里桥烧饼铺</t>
+          <t>杭州绿豆糕（河坊街）</t>
         </is>
       </c>
     </row>
@@ -2290,7 +2290,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>知味观</t>
+          <t>富春王记烧饼（中山中路店总店）</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>杭州绿豆糕（河坊街）</t>
+          <t>红帽叔叔包子</t>
         </is>
       </c>
     </row>
@@ -2314,7 +2314,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>富春王记烧饼（中山中路店总店）</t>
+          <t>潘老板炸鸡腿</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>红帽叔叔包子</t>
+          <t>熨斗大姐 葱包烩儿</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>潘老板炸鸡腿</t>
+          <t>新疆烤包子</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2350,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>熨斗大姐 葱包烩儿</t>
+          <t>李喜欢虾滑</t>
         </is>
       </c>
     </row>
@@ -2362,31 +2362,31 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>新疆烤包子</t>
+          <t>龙井茉莉花豆浆</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>李喜欢虾滑</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>龙井茉莉花豆浆</t>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -2398,7 +2398,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>王氏烧饼无矾油条</t>
         </is>
       </c>
     </row>
@@ -2410,31 +2410,31 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/16/2027</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>王氏烧饼无矾油条</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/16/2027</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -2445,30 +2445,6 @@
         </is>
       </c>
       <c r="B53" t="inlineStr">
-        <is>
-          <t>游埠豆浆（河坊街店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
         <is>
           <t>王氏烧饼无矾油条</t>
         </is>

</xml_diff>

<commit_message>
Day 2: 城隍庙豫园 in itinerary
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -699,7 +699,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">

</xml_diff>

<commit_message>
Day 2: dinner at 味香斋面馆
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -699,12 +699,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>外滩</t>
+          <t>晚餐 · 味香斋面馆（南京东路店）</t>
         </is>
       </c>
     </row>
@@ -716,12 +716,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>城隍庙 · 豫园</t>
+          <t>外滩</t>
         </is>
       </c>
     </row>
@@ -733,29 +733,29 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>城隍庙 · 豫园</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/09/2027</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>迪士尼小镇</t>
+          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>迪士尼小镇</t>
         </is>
       </c>
     </row>
@@ -784,12 +784,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>上海迪士尼乐园</t>
+          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -801,12 +801,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>迪士尼 · 跟拍（1 小时）</t>
+          <t>上海迪士尼乐园</t>
         </is>
       </c>
     </row>
@@ -818,12 +818,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>烟花 · 闭园</t>
+          <t>迪士尼 · 跟拍（1 小时）</t>
         </is>
       </c>
     </row>
@@ -835,29 +835,29 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>烟花 · 闭园</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>回酒店 · 嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>上海站</t>
+          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -886,12 +886,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>高铁 上海站 → 苏州站</t>
+          <t>上海站</t>
         </is>
       </c>
     </row>
@@ -903,12 +903,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>高铁 上海站 → 苏州站</t>
         </is>
       </c>
     </row>
@@ -920,12 +920,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>午餐 · 酒店附近</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -937,12 +937,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>虎丘风景区</t>
+          <t>午餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -954,12 +954,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>七里山塘千年古街</t>
+          <t>虎丘风景区</t>
         </is>
       </c>
     </row>
@@ -971,29 +971,29 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
+          <t>七里山塘千年古街</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>双塔市集</t>
+          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>双塔市集</t>
         </is>
       </c>
     </row>
@@ -1022,12 +1022,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>拙政园</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1039,12 +1039,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>狮子林</t>
+          <t>拙政园</t>
         </is>
       </c>
     </row>
@@ -1056,12 +1056,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>平江路</t>
+          <t>狮子林</t>
         </is>
       </c>
     </row>
@@ -1073,12 +1073,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>午餐 · 平江路</t>
+          <t>平江路</t>
         </is>
       </c>
     </row>
@@ -1090,12 +1090,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>月光码头</t>
+          <t>午餐 · 平江路</t>
         </is>
       </c>
     </row>
@@ -1107,12 +1107,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>金鸡湖 · 东方之门</t>
+          <t>月光码头</t>
         </is>
       </c>
     </row>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
+          <t>金鸡湖 · 东方之门</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1175,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>苏州 → 乌镇</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1192,12 +1192,12 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>苏州 → 乌镇</t>
         </is>
       </c>
     </row>
@@ -1209,12 +1209,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>半城红妆汉服体验店</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1226,12 +1226,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>乌镇景区</t>
+          <t>半城红妆汉服体验店</t>
         </is>
       </c>
     </row>
@@ -1243,29 +1243,29 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>回酒店 · 乌镇民宿</t>
+          <t>乌镇景区</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>早茶客 · 桥里桥烧饼铺</t>
+          <t>回酒店 · 乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>早茶客 · 桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -1294,12 +1294,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>乌镇 · 清晨漫步</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1311,12 +1311,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>午餐 · 退房</t>
+          <t>乌镇 · 清晨漫步</t>
         </is>
       </c>
     </row>
@@ -1328,12 +1328,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>乌镇 → 杭州</t>
+          <t>午餐 · 退房</t>
         </is>
       </c>
     </row>
@@ -1345,12 +1345,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>乌镇 → 杭州</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>钱王祠码头</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>三潭印月</t>
+          <t>钱王祠码头</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1396,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>三潭印月</t>
         </is>
       </c>
     </row>
@@ -1413,12 +1413,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>断桥残雪</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1430,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>武林夜市</t>
+          <t>断桥残雪</t>
         </is>
       </c>
     </row>
@@ -1447,29 +1447,29 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>武林夜市</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>上天竺法喜讲寺</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>灵隐寺</t>
+          <t>上天竺法喜讲寺</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>灵隐寺</t>
         </is>
       </c>
     </row>
@@ -1549,12 +1549,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>苏堤</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1566,12 +1566,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>太子湾公园</t>
+          <t>苏堤</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1583,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>雷峰塔</t>
+          <t>太子湾公园</t>
         </is>
       </c>
     </row>
@@ -1600,12 +1600,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>雷峰塔</t>
         </is>
       </c>
     </row>
@@ -1617,12 +1617,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>湖滨银泰 in77</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>湖滨银泰 in77</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>03/16/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>大马弄 · 南宋街 · 河坊街</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1702,12 +1702,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>大马弄 · 南宋街 · 河坊街</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>杭州东站</t>
+          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>上海南站</t>
+          <t>杭州东站</t>
         </is>
       </c>
     </row>
@@ -1753,12 +1753,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>景洪路站</t>
+          <t>上海南站</t>
         </is>
       </c>
     </row>
@@ -1770,12 +1770,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>上海浦东国际机场</t>
+          <t>景洪路站</t>
         </is>
       </c>
     </row>
@@ -1787,10 +1787,27 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
           <t>15:25</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>
@@ -1807,7 +1824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1918,7 +1935,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>德兴馆</t>
+          <t>味香斋面馆（南京东路店）</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1947,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>鲜得来排骨年糕（山西南路店）</t>
+          <t>沈大成</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1959,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>泸西老弄堂面馆</t>
+          <t>莱莱小笼包（南京东路店）</t>
         </is>
       </c>
     </row>
@@ -1954,31 +1971,31 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>沈大成</t>
+          <t>大壶春（四川中路店）</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>03/09/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>莱莱小笼包（南京东路店）</t>
+          <t>猪手饭（皮诺丘乡村厨房）</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>03/09/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>大壶春（四川中路店）</t>
+          <t>新旺茶餐室（迪士尼小镇）</t>
         </is>
       </c>
     </row>
@@ -1990,31 +2007,31 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>猪手饭（皮诺丘乡村厨房）</t>
+          <t>酸萝卜鸭腿（漫月出口餐车）</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>新旺茶餐室（迪士尼小镇）</t>
+          <t>万福兴（凤凰街店）</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>酸萝卜鸭腿（漫月出口餐车）</t>
+          <t>鑫震源 · 苏式大虾生煎</t>
         </is>
       </c>
     </row>
@@ -2026,7 +2043,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>万福兴（凤凰街店）</t>
+          <t>哑巴生煎（海市山塘 45 号）</t>
         </is>
       </c>
     </row>
@@ -2038,7 +2055,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>鑫震源 · 苏式大虾生煎</t>
+          <t>秋娟小吃店</t>
         </is>
       </c>
     </row>
@@ -2050,31 +2067,31 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>哑巴生煎（海市山塘 45 号）</t>
+          <t>沈万三 · 江南卤味（山塘街店）</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>秋娟小吃店</t>
+          <t>老客满蛋</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>沈万三 · 江南卤味（山塘街店）</t>
+          <t>大孃孃苏式糖水（双塔市集店）</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2103,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>老客满蛋</t>
+          <t>江南米造局（双塔市集店）</t>
         </is>
       </c>
     </row>
@@ -2098,7 +2115,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>大孃孃苏式糖水（双塔市集店）</t>
+          <t>苏拾里</t>
         </is>
       </c>
     </row>
@@ -2110,31 +2127,31 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>江南米造局（双塔市集店）</t>
+          <t>苏外婆</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>苏拾里</t>
+          <t>万福兴（凤凰街店）</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>苏外婆</t>
+          <t>鑫震源 · 苏式大虾生煎</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2163,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>万福兴（凤凰街店）</t>
+          <t>滋啦啦油煎铺</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2175,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>鑫震源 · 苏式大虾生煎</t>
+          <t>吴妈馄饨</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2187,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>滋啦啦油煎铺</t>
+          <t>锦记糕点铺</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2199,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>吴妈馄饨</t>
+          <t>书生羊肉面</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2211,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>锦记糕点铺</t>
+          <t>乌镇酱鸭店</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2223,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>书生羊肉面</t>
+          <t>永平粉团铺</t>
         </is>
       </c>
     </row>
@@ -2218,31 +2235,31 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>乌镇酱鸭店</t>
+          <t>锦岸私房菜</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>永平粉团铺</t>
+          <t>桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>锦岸私房菜</t>
+          <t>知味观</t>
         </is>
       </c>
     </row>
@@ -2254,7 +2271,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>桥里桥烧饼铺</t>
+          <t>杭州绿豆糕（河坊街）</t>
         </is>
       </c>
     </row>
@@ -2266,7 +2283,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>知味观</t>
+          <t>富春王记烧饼（中山中路店总店）</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2295,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>杭州绿豆糕（河坊街）</t>
+          <t>红帽叔叔包子</t>
         </is>
       </c>
     </row>
@@ -2290,7 +2307,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>富春王记烧饼（中山中路店总店）</t>
+          <t>潘老板炸鸡腿</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2319,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>红帽叔叔包子</t>
+          <t>熨斗大姐 葱包烩儿</t>
         </is>
       </c>
     </row>
@@ -2314,7 +2331,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>潘老板炸鸡腿</t>
+          <t>新疆烤包子</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2343,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>熨斗大姐 葱包烩儿</t>
+          <t>李喜欢虾滑</t>
         </is>
       </c>
     </row>
@@ -2338,31 +2355,31 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>新疆烤包子</t>
+          <t>龙井茉莉花豆浆</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>李喜欢虾滑</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>龙井茉莉花豆浆</t>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2391,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>王氏烧饼无矾油条</t>
         </is>
       </c>
     </row>
@@ -2386,31 +2403,31 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/16/2027</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>王氏烧饼无矾油条</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/16/2027</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -2421,30 +2438,6 @@
         </is>
       </c>
       <c r="B51" t="inlineStr">
-        <is>
-          <t>游埠豆浆（河坊街店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
         <is>
           <t>王氏烧饼无矾油条</t>
         </is>

</xml_diff>

<commit_message>
Day 2: 外滩 before dinner
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -699,12 +699,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>晚餐 · 味香斋面馆（南京东路店）</t>
+          <t>外滩</t>
         </is>
       </c>
     </row>
@@ -716,12 +716,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:45</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>外滩</t>
+          <t>晚餐 · 味香斋面馆（南京东路店）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix hotel exit sorting before same-time first stop
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -767,12 +767,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>迪士尼小镇</t>
+          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>嘉虹酒店（上海浦东机场川沙地铁站店）</t>
+          <t>迪士尼小镇</t>
         </is>
       </c>
     </row>
@@ -1005,12 +1005,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:50</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>双塔市集</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>双塔市集</t>
         </is>
       </c>
     </row>
@@ -1158,12 +1158,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1277,12 +1277,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:50</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>早茶客 · 桥里桥烧饼铺</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1299,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>早茶客 · 桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1503,7 +1503,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day 4: lunch at 万福兴
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>午餐 · 酒店附近</t>
+          <t>午餐 · 万福兴（凤凰街店）</t>
         </is>
       </c>
     </row>
@@ -1824,7 +1824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>鑫震源 · 苏式大虾生煎</t>
+          <t>哑巴生煎（海市山塘 45 号）</t>
         </is>
       </c>
     </row>
@@ -2043,7 +2043,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>哑巴生煎（海市山塘 45 号）</t>
+          <t>秋娟小吃店</t>
         </is>
       </c>
     </row>
@@ -2055,19 +2055,19 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>秋娟小吃店</t>
+          <t>沈万三 · 江南卤味（山塘街店）</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>沈万三 · 江南卤味（山塘街店）</t>
+          <t>老客满蛋</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2079,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>老客满蛋</t>
+          <t>大孃孃苏式糖水（双塔市集店）</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>大孃孃苏式糖水（双塔市集店）</t>
+          <t>江南米造局（双塔市集店）</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>江南米造局（双塔市集店）</t>
+          <t>苏拾里</t>
         </is>
       </c>
     </row>
@@ -2115,19 +2115,19 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>苏拾里</t>
+          <t>苏外婆</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>苏外婆</t>
+          <t>万福兴（凤凰街店）</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>万福兴（凤凰街店）</t>
+          <t>鑫震源 · 苏式大虾生煎</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>鑫震源 · 苏式大虾生煎</t>
+          <t>滋啦啦油煎铺</t>
         </is>
       </c>
     </row>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>滋啦啦油煎铺</t>
+          <t>吴妈馄饨</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>吴妈馄饨</t>
+          <t>锦记糕点铺</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>锦记糕点铺</t>
+          <t>书生羊肉面</t>
         </is>
       </c>
     </row>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>书生羊肉面</t>
+          <t>乌镇酱鸭店</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>乌镇酱鸭店</t>
+          <t>永平粉团铺</t>
         </is>
       </c>
     </row>
@@ -2223,19 +2223,19 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>永平粉团铺</t>
+          <t>锦岸私房菜</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>锦岸私房菜</t>
+          <t>桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>桥里桥烧饼铺</t>
+          <t>知味观</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>知味观</t>
+          <t>杭州绿豆糕（河坊街）</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>杭州绿豆糕（河坊街）</t>
+          <t>富春王记烧饼（中山中路店总店）</t>
         </is>
       </c>
     </row>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>富春王记烧饼（中山中路店总店）</t>
+          <t>红帽叔叔包子</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2295,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>红帽叔叔包子</t>
+          <t>潘老板炸鸡腿</t>
         </is>
       </c>
     </row>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>潘老板炸鸡腿</t>
+          <t>熨斗大姐 葱包烩儿</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>熨斗大姐 葱包烩儿</t>
+          <t>新疆烤包子</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>新疆烤包子</t>
+          <t>李喜欢虾滑</t>
         </is>
       </c>
     </row>
@@ -2343,19 +2343,19 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>李喜欢虾滑</t>
+          <t>龙井茉莉花豆浆</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>龙井茉莉花豆浆</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
+          <t>王氏烧饼无矾油条</t>
         </is>
       </c>
     </row>
@@ -2391,19 +2391,19 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>王氏烧饼无矾油条</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/16/2027</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -2415,7 +2415,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -2426,18 +2426,6 @@
         </is>
       </c>
       <c r="B50" t="inlineStr">
-        <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
         <is>
           <t>王氏烧饼无矾油条</t>
         </is>

</xml_diff>

<commit_message>
Day 4: dinner at 沈万三
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -988,29 +988,29 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
+          <t>晚餐 · 沈万三 · 江南卤味（山塘街店）</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>08:50</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1022,12 +1022,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:50</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>双塔市集</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1039,12 +1039,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>拙政园</t>
+          <t>双塔市集</t>
         </is>
       </c>
     </row>
@@ -1056,12 +1056,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>狮子林</t>
+          <t>拙政园</t>
         </is>
       </c>
     </row>
@@ -1073,12 +1073,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>平江路</t>
+          <t>狮子林</t>
         </is>
       </c>
     </row>
@@ -1090,12 +1090,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>午餐 · 平江路</t>
+          <t>平江路</t>
         </is>
       </c>
     </row>
@@ -1107,12 +1107,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>月光码头</t>
+          <t>午餐 · 平江路</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1124,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>金鸡湖 · 东方之门</t>
+          <t>月光码头</t>
         </is>
       </c>
     </row>
@@ -1141,29 +1141,29 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
+          <t>金鸡湖 · 东方之门</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1175,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1192,12 +1192,12 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>苏州 → 乌镇</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1209,12 +1209,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>苏州 → 乌镇</t>
         </is>
       </c>
     </row>
@@ -1226,12 +1226,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>半城红妆汉服体验店</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1243,12 +1243,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>乌镇景区</t>
+          <t>半城红妆汉服体验店</t>
         </is>
       </c>
     </row>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>回酒店 · 乌镇民宿</t>
+          <t>乌镇景区</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>06:50</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>回酒店 · 乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1294,12 +1294,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:50</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>早茶客 · 桥里桥烧饼铺</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1311,12 +1311,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>乌镇 · 清晨漫步</t>
+          <t>早茶客 · 桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -1328,12 +1328,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>午餐 · 退房</t>
+          <t>乌镇 · 清晨漫步</t>
         </is>
       </c>
     </row>
@@ -1345,12 +1345,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>乌镇 → 杭州</t>
+          <t>午餐 · 退房</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>乌镇 → 杭州</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>钱王祠码头</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1396,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>三潭印月</t>
+          <t>钱王祠码头</t>
         </is>
       </c>
     </row>
@@ -1413,12 +1413,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>三潭印月</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1430,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>断桥残雪</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1447,12 +1447,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>武林夜市</t>
+          <t>断桥残雪</t>
         </is>
       </c>
     </row>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>武林夜市</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>上天竺法喜讲寺</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>灵隐寺</t>
+          <t>上天竺法喜讲寺</t>
         </is>
       </c>
     </row>
@@ -1549,12 +1549,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>灵隐寺</t>
         </is>
       </c>
     </row>
@@ -1566,12 +1566,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>苏堤</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1583,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>太子湾公园</t>
+          <t>苏堤</t>
         </is>
       </c>
     </row>
@@ -1600,12 +1600,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>雷峰塔</t>
+          <t>太子湾公园</t>
         </is>
       </c>
     </row>
@@ -1617,12 +1617,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>雷峰塔</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>湖滨银泰 in77</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
@@ -1651,29 +1651,29 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>湖滨银泰 in77</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>03/16/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1702,12 +1702,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>大马弄 · 南宋街 · 河坊街</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>大马弄 · 南宋街 · 河坊街</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>杭州东站</t>
+          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1753,12 +1753,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>上海南站</t>
+          <t>杭州东站</t>
         </is>
       </c>
     </row>
@@ -1770,12 +1770,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>景洪路站</t>
+          <t>上海南站</t>
         </is>
       </c>
     </row>
@@ -1787,12 +1787,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>上海浦东国际机场</t>
+          <t>景洪路站</t>
         </is>
       </c>
     </row>
@@ -1804,10 +1804,27 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
           <t>15:25</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C82" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>

</xml_diff>

<commit_message>
Day 5: lunch at 苏外婆
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -1112,7 +1112,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>午餐 · 平江路</t>
+          <t>午餐 · 苏外婆（平江路总店）</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2120,19 +2120,19 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>苏拾里</t>
+          <t>苏外婆 · 苏帮菜 · 松鼠桂鱼（平江路总店）</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>苏外婆</t>
+          <t>万福兴（凤凰街店）</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2144,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>万福兴（凤凰街店）</t>
+          <t>鑫震源 · 苏式大虾生煎</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>鑫震源 · 苏式大虾生煎</t>
+          <t>滋啦啦油煎铺</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>滋啦啦油煎铺</t>
+          <t>吴妈馄饨</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>吴妈馄饨</t>
+          <t>锦记糕点铺</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>锦记糕点铺</t>
+          <t>书生羊肉面</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>书生羊肉面</t>
+          <t>乌镇酱鸭店</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>乌镇酱鸭店</t>
+          <t>永平粉团铺</t>
         </is>
       </c>
     </row>
@@ -2228,19 +2228,19 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>永平粉团铺</t>
+          <t>锦岸私房菜</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>锦岸私房菜</t>
+          <t>桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>桥里桥烧饼铺</t>
+          <t>知味观</t>
         </is>
       </c>
     </row>
@@ -2264,7 +2264,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>知味观</t>
+          <t>杭州绿豆糕（河坊街）</t>
         </is>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>杭州绿豆糕（河坊街）</t>
+          <t>富春王记烧饼（中山中路店总店）</t>
         </is>
       </c>
     </row>
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>富春王记烧饼（中山中路店总店）</t>
+          <t>红帽叔叔包子</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>红帽叔叔包子</t>
+          <t>潘老板炸鸡腿</t>
         </is>
       </c>
     </row>
@@ -2312,7 +2312,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>潘老板炸鸡腿</t>
+          <t>熨斗大姐 葱包烩儿</t>
         </is>
       </c>
     </row>
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>熨斗大姐 葱包烩儿</t>
+          <t>新疆烤包子</t>
         </is>
       </c>
     </row>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>新疆烤包子</t>
+          <t>李喜欢虾滑</t>
         </is>
       </c>
     </row>
@@ -2348,19 +2348,19 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>李喜欢虾滑</t>
+          <t>龙井茉莉花豆浆</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>龙井茉莉花豆浆</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -2372,7 +2372,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
+          <t>王氏烧饼无矾油条</t>
         </is>
       </c>
     </row>
@@ -2396,19 +2396,19 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>王氏烧饼无矾油条</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/16/2027</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -2420,7 +2420,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -2431,18 +2431,6 @@
         </is>
       </c>
       <c r="B49" t="inlineStr">
-        <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
         <is>
           <t>王氏烧饼无矾油条</t>
         </is>

</xml_diff>

<commit_message>
Day 6: breakfast at 鑫震源
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -1197,7 +1197,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>早餐 · 鑫震源（大儒巷店）</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>万福兴（凤凰街店）</t>
+          <t>鑫震源 · 苏式大虾生煎（大儒巷店）</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2144,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>鑫震源 · 苏式大虾生煎</t>
+          <t>滋啦啦油煎铺</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>滋啦啦油煎铺</t>
+          <t>吴妈馄饨</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>吴妈馄饨</t>
+          <t>锦记糕点铺</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>锦记糕点铺</t>
+          <t>书生羊肉面</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>书生羊肉面</t>
+          <t>乌镇酱鸭店</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>乌镇酱鸭店</t>
+          <t>永平粉团铺</t>
         </is>
       </c>
     </row>
@@ -2216,19 +2216,19 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>永平粉团铺</t>
+          <t>锦岸私房菜</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>锦岸私房菜</t>
+          <t>桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>桥里桥烧饼铺</t>
+          <t>知味观</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>知味观</t>
+          <t>杭州绿豆糕（河坊街）</t>
         </is>
       </c>
     </row>
@@ -2264,7 +2264,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>杭州绿豆糕（河坊街）</t>
+          <t>富春王记烧饼（中山中路店总店）</t>
         </is>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>富春王记烧饼（中山中路店总店）</t>
+          <t>红帽叔叔包子</t>
         </is>
       </c>
     </row>
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>红帽叔叔包子</t>
+          <t>潘老板炸鸡腿</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>潘老板炸鸡腿</t>
+          <t>熨斗大姐 葱包烩儿</t>
         </is>
       </c>
     </row>
@@ -2312,7 +2312,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>熨斗大姐 葱包烩儿</t>
+          <t>新疆烤包子</t>
         </is>
       </c>
     </row>
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>新疆烤包子</t>
+          <t>李喜欢虾滑</t>
         </is>
       </c>
     </row>
@@ -2336,19 +2336,19 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>李喜欢虾滑</t>
+          <t>龙井茉莉花豆浆</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>龙井茉莉花豆浆</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -2372,7 +2372,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
+          <t>王氏烧饼无矾油条</t>
         </is>
       </c>
     </row>
@@ -2384,19 +2384,19 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>王氏烧饼无矾油条</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/16/2027</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -2419,18 +2419,6 @@
         </is>
       </c>
       <c r="B48" t="inlineStr">
-        <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
         <is>
           <t>王氏烧饼无矾油条</t>
         </is>

</xml_diff>

<commit_message>
Day 6: lunch at 书生羊肉面
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1277,29 +1277,29 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>回酒店 · 乌镇民宿</t>
+          <t>午餐 · 书生羊肉面</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>06:50</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>回酒店 · 乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1311,12 +1311,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:50</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>早茶客 · 桥里桥烧饼铺</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1328,12 +1328,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>乌镇 · 清晨漫步</t>
+          <t>早茶客 · 桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -1345,12 +1345,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>午餐 · 退房</t>
+          <t>乌镇 · 清晨漫步</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>乌镇 → 杭州</t>
+          <t>午餐 · 退房</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>乌镇 → 杭州</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1396,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>钱王祠码头</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1413,12 +1413,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>三潭印月</t>
+          <t>钱王祠码头</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1430,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>三潭印月</t>
         </is>
       </c>
     </row>
@@ -1447,12 +1447,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>断桥残雪</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1464,12 +1464,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>武林夜市</t>
+          <t>断桥残雪</t>
         </is>
       </c>
     </row>
@@ -1481,29 +1481,29 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>武林夜市</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>上天竺法喜讲寺</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1549,12 +1549,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>灵隐寺</t>
+          <t>上天竺法喜讲寺</t>
         </is>
       </c>
     </row>
@@ -1566,12 +1566,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>灵隐寺</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1583,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>苏堤</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1600,12 +1600,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>太子湾公园</t>
+          <t>苏堤</t>
         </is>
       </c>
     </row>
@@ -1617,12 +1617,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>雷峰塔</t>
+          <t>太子湾公园</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>雷峰塔</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1651,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>湖滨银泰 in77</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
@@ -1668,29 +1668,29 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>湖滨银泰 in77</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>03/16/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1702,12 +1702,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>大马弄 · 南宋街 · 河坊街</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>大马弄 · 南宋街 · 河坊街</t>
         </is>
       </c>
     </row>
@@ -1753,12 +1753,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>杭州东站</t>
+          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1770,12 +1770,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>上海南站</t>
+          <t>杭州东站</t>
         </is>
       </c>
     </row>
@@ -1787,12 +1787,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>景洪路站</t>
+          <t>上海南站</t>
         </is>
       </c>
     </row>
@@ -1804,12 +1804,12 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>上海浦东国际机场</t>
+          <t>景洪路站</t>
         </is>
       </c>
     </row>
@@ -1821,10 +1821,27 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
           <t>15:25</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>
@@ -1841,7 +1858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2156,7 +2173,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>吴妈馄饨</t>
+          <t>锦记糕点铺</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2185,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>锦记糕点铺</t>
+          <t>书生羊肉面</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2197,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>书生羊肉面</t>
+          <t>永平粉团铺</t>
         </is>
       </c>
     </row>
@@ -2192,31 +2209,31 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>乌镇酱鸭店</t>
+          <t>锦岸私房菜</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>永平粉团铺</t>
+          <t>桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>锦岸私房菜</t>
+          <t>知味观</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2245,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>桥里桥烧饼铺</t>
+          <t>杭州绿豆糕（河坊街）</t>
         </is>
       </c>
     </row>
@@ -2240,7 +2257,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>知味观</t>
+          <t>富春王记烧饼（中山中路店总店）</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2269,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>杭州绿豆糕（河坊街）</t>
+          <t>红帽叔叔包子</t>
         </is>
       </c>
     </row>
@@ -2264,7 +2281,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>富春王记烧饼（中山中路店总店）</t>
+          <t>潘老板炸鸡腿</t>
         </is>
       </c>
     </row>
@@ -2276,7 +2293,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>红帽叔叔包子</t>
+          <t>熨斗大姐 葱包烩儿</t>
         </is>
       </c>
     </row>
@@ -2288,7 +2305,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>潘老板炸鸡腿</t>
+          <t>新疆烤包子</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2317,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>熨斗大姐 葱包烩儿</t>
+          <t>李喜欢虾滑</t>
         </is>
       </c>
     </row>
@@ -2312,31 +2329,31 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>新疆烤包子</t>
+          <t>龙井茉莉花豆浆</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>李喜欢虾滑</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>龙井茉莉花豆浆</t>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2365,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>王氏烧饼无矾油条</t>
         </is>
       </c>
     </row>
@@ -2360,31 +2377,31 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/16/2027</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>王氏烧饼无矾油条</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/16/2027</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -2395,30 +2412,6 @@
         </is>
       </c>
       <c r="B46" t="inlineStr">
-        <is>
-          <t>游埠豆浆（河坊街店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
         <is>
           <t>王氏烧饼无矾油条</t>
         </is>

</xml_diff>

<commit_message>
Day 6: dinner at 锦岸私房菜
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>回酒店 · 乌镇民宿</t>
+          <t>晚餐 · 锦岸私房菜</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>06:50</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>回酒店 · 乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1328,12 +1328,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:50</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>早茶客 · 桥里桥烧饼铺</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1345,12 +1345,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>乌镇 · 清晨漫步</t>
+          <t>早茶客 · 桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>午餐 · 退房</t>
+          <t>乌镇 · 清晨漫步</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>乌镇 → 杭州</t>
+          <t>午餐 · 退房</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1396,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>乌镇 → 杭州</t>
         </is>
       </c>
     </row>
@@ -1413,12 +1413,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>钱王祠码头</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1430,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>三潭印月</t>
+          <t>钱王祠码头</t>
         </is>
       </c>
     </row>
@@ -1447,12 +1447,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>三潭印月</t>
         </is>
       </c>
     </row>
@@ -1464,12 +1464,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>断桥残雪</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>武林夜市</t>
+          <t>断桥残雪</t>
         </is>
       </c>
     </row>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>武林夜市</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1549,12 +1549,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>上天竺法喜讲寺</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1566,12 +1566,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>灵隐寺</t>
+          <t>上天竺法喜讲寺</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1583,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>灵隐寺</t>
         </is>
       </c>
     </row>
@@ -1600,12 +1600,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>苏堤</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1617,12 +1617,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>太子湾公园</t>
+          <t>苏堤</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>雷峰塔</t>
+          <t>太子湾公园</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1651,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>雷峰塔</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>湖滨银泰 in77</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
@@ -1685,29 +1685,29 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>湖滨银泰 in77</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>03/16/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>大马弄 · 南宋街 · 河坊街</t>
+          <t>早餐 · 酒店附近</t>
         </is>
       </c>
     </row>
@@ -1753,12 +1753,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>大马弄 · 南宋街 · 河坊街</t>
         </is>
       </c>
     </row>
@@ -1770,12 +1770,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>杭州东站</t>
+          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1787,12 +1787,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>上海南站</t>
+          <t>杭州东站</t>
         </is>
       </c>
     </row>
@@ -1804,12 +1804,12 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>景洪路站</t>
+          <t>上海南站</t>
         </is>
       </c>
     </row>
@@ -1821,12 +1821,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>上海浦东国际机场</t>
+          <t>景洪路站</t>
         </is>
       </c>
     </row>
@@ -1838,10 +1838,27 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
           <t>15:25</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>

</xml_diff>

<commit_message>
Day 8 breakfast/dinner, Day 9 breakfast
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -1554,7 +1554,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>早餐 · 游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>晚餐 · 杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>早餐 · 酒店附近</t>
+          <t>早餐 · 泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -1875,7 +1875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2370,67 +2370,19 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
+          <t>杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/16/2027</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>王氏烧饼无矾油条</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>03/15/2027</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>杭州酒家（延安路店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>游埠豆浆（河坊街店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
           <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>03/16/2027</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>王氏烧饼无矾油条</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day 7: leave Wuzhen earlier
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>午餐 · 退房</t>
+          <t>退房 · 乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1430,12 +1430,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>钱王祠码头</t>
+          <t>午餐 · 河坊街</t>
         </is>
       </c>
     </row>
@@ -1447,12 +1447,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>三潭印月</t>
+          <t>钱王祠码头</t>
         </is>
       </c>
     </row>
@@ -1464,12 +1464,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>三潭印月</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>断桥残雪</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>武林夜市</t>
+          <t>断桥残雪</t>
         </is>
       </c>
     </row>
@@ -1515,29 +1515,29 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>武林夜市</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1549,12 +1549,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>早餐 · 游埠豆浆（河坊街店）</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1566,12 +1566,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>上天竺法喜讲寺</t>
+          <t>早餐 · 游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1583,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>灵隐寺</t>
+          <t>上天竺法喜讲寺</t>
         </is>
       </c>
     </row>
@@ -1600,12 +1600,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>灵隐寺</t>
         </is>
       </c>
     </row>
@@ -1617,12 +1617,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>苏堤</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>太子湾公园</t>
+          <t>苏堤</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1651,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>雷峰塔</t>
+          <t>太子湾公园</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>晚餐 · 杭州酒家（延安路店）</t>
+          <t>雷峰塔</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>湖滨银泰 in77</t>
+          <t>晚餐 · 杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
@@ -1702,29 +1702,29 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>湖滨银泰 in77</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>03/16/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>早餐 · 泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1753,12 +1753,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>大马弄 · 南宋街 · 河坊街</t>
+          <t>早餐 · 泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -1770,12 +1770,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>大马弄 · 南宋街 · 河坊街</t>
         </is>
       </c>
     </row>
@@ -1787,12 +1787,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>杭州东站</t>
+          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1804,12 +1804,12 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>上海南站</t>
+          <t>杭州东站</t>
         </is>
       </c>
     </row>
@@ -1821,12 +1821,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>景洪路站</t>
+          <t>上海南站</t>
         </is>
       </c>
     </row>
@@ -1838,12 +1838,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>上海浦东国际机场</t>
+          <t>景洪路站</t>
         </is>
       </c>
     </row>
@@ -1855,10 +1855,27 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
           <t>15:25</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>

</xml_diff>

<commit_message>
Day 7: lunch at 赵府私厨
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -1435,7 +1435,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>午餐 · 河坊街</t>
+          <t>午餐 · 赵府私厨 · 老杭帮菜（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>知味观</t>
+          <t>赵府私厨 · 老杭帮菜（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>杭州绿豆糕（河坊街）</t>
+          <t>知味观</t>
         </is>
       </c>
     </row>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>富春王记烧饼（中山中路店总店）</t>
+          <t>杭州绿豆糕（河坊街）</t>
         </is>
       </c>
     </row>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>红帽叔叔包子</t>
+          <t>富春王记烧饼（中山中路店总店）</t>
         </is>
       </c>
     </row>
@@ -2315,7 +2315,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>潘老板炸鸡腿</t>
+          <t>红帽叔叔包子</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>熨斗大姐 葱包烩儿</t>
+          <t>潘老板炸鸡腿</t>
         </is>
       </c>
     </row>
@@ -2339,7 +2339,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>新疆烤包子</t>
+          <t>熨斗大姐 葱包烩儿</t>
         </is>
       </c>
     </row>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>李喜欢虾滑</t>
+          <t>新疆烤包子</t>
         </is>
       </c>
     </row>
@@ -2363,19 +2363,19 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>龙井茉莉花豆浆</t>
+          <t>李喜欢虾滑</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>龙井茉莉花豆浆</t>
         </is>
       </c>
     </row>
@@ -2387,17 +2387,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>杭州酒家（延安路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
           <t>03/16/2027</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>

</xml_diff>

<commit_message>
Day 7: 河坊街 in afternoon
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1447,12 +1447,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>钱王祠码头</t>
+          <t>河坊街</t>
         </is>
       </c>
     </row>
@@ -1464,12 +1464,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>三潭印月</t>
+          <t>钱王祠码头</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>三潭印月</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>断桥残雪</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>武林夜市</t>
+          <t>断桥残雪</t>
         </is>
       </c>
     </row>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>武林夜市</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1566,12 +1566,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>早餐 · 游埠豆浆（河坊街店）</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1583,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>上天竺法喜讲寺</t>
+          <t>早餐 · 游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1600,12 +1600,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>灵隐寺</t>
+          <t>上天竺法喜讲寺</t>
         </is>
       </c>
     </row>
@@ -1617,12 +1617,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>灵隐寺</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>苏堤</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1651,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>太子湾公园</t>
+          <t>苏堤</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>雷峰塔</t>
+          <t>太子湾公园</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>晚餐 · 杭州酒家（延安路店）</t>
+          <t>雷峰塔</t>
         </is>
       </c>
     </row>
@@ -1702,12 +1702,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>湖滨银泰 in77</t>
+          <t>晚餐 · 杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
@@ -1719,29 +1719,29 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>湖滨银泰 in77</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>03/16/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1753,12 +1753,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>早餐 · 泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1770,12 +1770,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>大马弄 · 南宋街 · 河坊街</t>
+          <t>早餐 · 泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -1787,12 +1787,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>大马弄 · 南宋街 · 河坊街</t>
         </is>
       </c>
     </row>
@@ -1804,12 +1804,12 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>杭州东站</t>
+          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1821,12 +1821,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>上海南站</t>
+          <t>杭州东站</t>
         </is>
       </c>
     </row>
@@ -1838,12 +1838,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>景洪路站</t>
+          <t>上海南站</t>
         </is>
       </c>
     </row>
@@ -1855,12 +1855,12 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>上海浦东国际机场</t>
+          <t>景洪路站</t>
         </is>
       </c>
     </row>
@@ -1872,10 +1872,27 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
           <t>15:25</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>

</xml_diff>

<commit_message>
Day 6: return hanfu in the evening
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1311,29 +1311,29 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>回酒店 · 乌镇民宿</t>
+          <t>还汉服 · 半城红妆汉服体验店</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>06:50</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>回酒店 · 乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1345,12 +1345,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:50</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>早茶客 · 桥里桥烧饼铺</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>乌镇 · 清晨漫步</t>
+          <t>早茶客 · 桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>退房 · 乌镇民宿</t>
+          <t>乌镇 · 清晨漫步</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1396,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>乌镇 → 杭州</t>
+          <t>退房 · 乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1413,12 +1413,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>乌镇 → 杭州</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1430,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>午餐 · 赵府私厨 · 老杭帮菜（河坊街店）</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1447,12 +1447,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>河坊街</t>
+          <t>午餐 · 赵府私厨 · 老杭帮菜（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1464,12 +1464,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>钱王祠码头</t>
+          <t>河坊街</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>三潭印月</t>
+          <t>钱王祠码头</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>三潭印月</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>断桥残雪</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>武林夜市</t>
+          <t>断桥残雪</t>
         </is>
       </c>
     </row>
@@ -1549,29 +1549,29 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>武林夜市</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1583,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>早餐 · 游埠豆浆（河坊街店）</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1600,12 +1600,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>上天竺法喜讲寺</t>
+          <t>早餐 · 游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1617,12 +1617,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>灵隐寺</t>
+          <t>上天竺法喜讲寺</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>灵隐寺</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1651,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>苏堤</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>太子湾公园</t>
+          <t>苏堤</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>雷峰塔</t>
+          <t>太子湾公园</t>
         </is>
       </c>
     </row>
@@ -1702,12 +1702,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>晚餐 · 杭州酒家（延安路店）</t>
+          <t>雷峰塔</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>湖滨银泰 in77</t>
+          <t>晚餐 · 杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
@@ -1736,29 +1736,29 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>湖滨银泰 in77</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>03/16/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1770,12 +1770,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>早餐 · 泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1787,12 +1787,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>大马弄 · 南宋街 · 河坊街</t>
+          <t>早餐 · 泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -1804,12 +1804,12 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>大马弄 · 南宋街 · 河坊街</t>
         </is>
       </c>
     </row>
@@ -1821,12 +1821,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>杭州东站</t>
+          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1838,12 +1838,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>上海南站</t>
+          <t>杭州东站</t>
         </is>
       </c>
     </row>
@@ -1855,12 +1855,12 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>景洪路站</t>
+          <t>上海南站</t>
         </is>
       </c>
     </row>
@@ -1872,12 +1872,12 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>上海浦东国际机场</t>
+          <t>景洪路站</t>
         </is>
       </c>
     </row>
@@ -1889,10 +1889,27 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
           <t>15:25</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>

</xml_diff>

<commit_message>
Day 5: dinner at 新梅华, 松鹤楼 in food tab
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
+          <t>晚餐 · 新梅华 · 非遗苏帮菜（星悦汇店）</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>行乐酒店（苏州观前街平江路店）</t>
+          <t>回酒店 · 行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1192,12 +1192,12 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>早餐 · 鑫震源（大儒巷店）</t>
+          <t>行乐酒店（苏州观前街平江路店）</t>
         </is>
       </c>
     </row>
@@ -1209,12 +1209,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>苏州 → 乌镇</t>
+          <t>早餐 · 鑫震源（大儒巷店）</t>
         </is>
       </c>
     </row>
@@ -1226,12 +1226,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>苏州 → 乌镇</t>
         </is>
       </c>
     </row>
@@ -1243,12 +1243,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>半城红妆汉服体验店</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1260,12 +1260,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>乌镇景区</t>
+          <t>半城红妆汉服体验店</t>
         </is>
       </c>
     </row>
@@ -1277,12 +1277,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>午餐 · 书生羊肉面</t>
+          <t>乌镇景区</t>
         </is>
       </c>
     </row>
@@ -1294,12 +1294,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>晚餐 · 锦岸私房菜</t>
+          <t>午餐 · 书生羊肉面</t>
         </is>
       </c>
     </row>
@@ -1311,12 +1311,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>还汉服 · 半城红妆汉服体验店</t>
+          <t>晚餐 · 锦岸私房菜</t>
         </is>
       </c>
     </row>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>回酒店 · 乌镇民宿</t>
+          <t>还汉服 · 半城红妆汉服体验店</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>06:50</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>乌镇民宿</t>
+          <t>回酒店 · 乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:50</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>早茶客 · 桥里桥烧饼铺</t>
+          <t>乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>乌镇 · 清晨漫步</t>
+          <t>早茶客 · 桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1396,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>退房 · 乌镇民宿</t>
+          <t>乌镇 · 清晨漫步</t>
         </is>
       </c>
     </row>
@@ -1413,12 +1413,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>乌镇 → 杭州</t>
+          <t>退房 · 乌镇民宿</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1430,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>乌镇 → 杭州</t>
         </is>
       </c>
     </row>
@@ -1447,12 +1447,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>午餐 · 赵府私厨 · 老杭帮菜（河坊街店）</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1464,12 +1464,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>河坊街</t>
+          <t>午餐 · 赵府私厨 · 老杭帮菜（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>钱王祠码头</t>
+          <t>河坊街</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>三潭印月</t>
+          <t>钱王祠码头</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>三潭印月</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>断桥残雪</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1549,12 +1549,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>武林夜市</t>
+          <t>断桥残雪</t>
         </is>
       </c>
     </row>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>武林夜市</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1600,12 +1600,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>早餐 · 游埠豆浆（河坊街店）</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1617,12 +1617,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>上天竺法喜讲寺</t>
+          <t>早餐 · 游埠豆浆（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>灵隐寺</t>
+          <t>上天竺法喜讲寺</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1651,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>曲院风荷</t>
+          <t>灵隐寺</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>苏堤</t>
+          <t>曲院风荷</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>太子湾公园</t>
+          <t>苏堤</t>
         </is>
       </c>
     </row>
@@ -1702,12 +1702,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>雷峰塔</t>
+          <t>太子湾公园</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>晚餐 · 杭州酒家（延安路店）</t>
+          <t>雷峰塔</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>湖滨银泰 in77</t>
+          <t>晚餐 · 杭州酒家（延安路店）</t>
         </is>
       </c>
     </row>
@@ -1753,29 +1753,29 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>湖滨银泰 in77</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>03/16/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>回酒店 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1787,12 +1787,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>早餐 · 泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
+          <t>嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1804,12 +1804,12 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>大马弄 · 南宋街 · 河坊街</t>
+          <t>早餐 · 泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>
       </c>
     </row>
@@ -1821,12 +1821,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
+          <t>大马弄 · 南宋街 · 河坊街</t>
         </is>
       </c>
     </row>
@@ -1838,12 +1838,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>杭州东站</t>
+          <t>回酒店退房 · 嘉虹酒店（杭州西湖河坊街店）</t>
         </is>
       </c>
     </row>
@@ -1855,12 +1855,12 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>上海南站</t>
+          <t>杭州东站</t>
         </is>
       </c>
     </row>
@@ -1872,12 +1872,12 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>景洪路站</t>
+          <t>上海南站</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>上海浦东国际机场</t>
+          <t>景洪路站</t>
         </is>
       </c>
     </row>
@@ -1906,10 +1906,27 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>上海浦东国际机场</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>03/16/2027</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
           <t>15:25</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>航班 MH389 上海 → 吉隆坡</t>
         </is>
@@ -1926,7 +1943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2212,24 +2229,24 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>鑫震源 · 苏式大虾生煎（大儒巷店）</t>
+          <t>新梅华 · 非遗苏帮菜（星悦汇店）</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>滋啦啦油煎铺</t>
+          <t>松鹤楼（苏州中心商场店）</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2258,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>锦记糕点铺</t>
+          <t>鑫震源 · 苏式大虾生煎（大儒巷店）</t>
         </is>
       </c>
     </row>
@@ -2253,7 +2270,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>书生羊肉面</t>
+          <t>滋啦啦油煎铺</t>
         </is>
       </c>
     </row>
@@ -2265,7 +2282,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>永平粉团铺</t>
+          <t>锦记糕点铺</t>
         </is>
       </c>
     </row>
@@ -2277,31 +2294,31 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>锦岸私房菜</t>
+          <t>书生羊肉面</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>桥里桥烧饼铺</t>
+          <t>永平粉团铺</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>赵府私厨 · 老杭帮菜（河坊街店）</t>
+          <t>锦岸私房菜</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2330,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>知味观</t>
+          <t>桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2342,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>杭州绿豆糕（河坊街）</t>
+          <t>赵府私厨 · 老杭帮菜（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -2337,7 +2354,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>富春王记烧饼（中山中路店总店）</t>
+          <t>知味观</t>
         </is>
       </c>
     </row>
@@ -2349,7 +2366,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>红帽叔叔包子</t>
+          <t>杭州绿豆糕（河坊街）</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2378,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>潘老板炸鸡腿</t>
+          <t>富春王记烧饼（中山中路店总店）</t>
         </is>
       </c>
     </row>
@@ -2373,7 +2390,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>熨斗大姐 葱包烩儿</t>
+          <t>红帽叔叔包子</t>
         </is>
       </c>
     </row>
@@ -2385,7 +2402,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>新疆烤包子</t>
+          <t>潘老板炸鸡腿</t>
         </is>
       </c>
     </row>
@@ -2397,7 +2414,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>李喜欢虾滑</t>
+          <t>熨斗大姐 葱包烩儿</t>
         </is>
       </c>
     </row>
@@ -2409,41 +2426,65 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>龙井茉莉花豆浆</t>
+          <t>新疆烤包子</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>李喜欢虾滑</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>龙井茉莉花豆浆</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>游埠豆浆（河坊街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>杭州酒家（延安路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
           <t>03/16/2027</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>

</xml_diff>

<commit_message>
Food tab: backup lunch/dinner per day
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -1943,7 +1943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2037,12 +2037,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>03/09/2027</t>
+          <t>03/08/2027</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>莱莱小笼（乔艾静安店）</t>
+          <t>和满堂 · 经典本帮菜</t>
         </is>
       </c>
     </row>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>味香斋面馆（南京东路店）</t>
+          <t>莱莱小笼（乔艾静安店）</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>沈大成</t>
+          <t>味香斋面馆（南京东路店）</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2078,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>莱莱小笼包（南京东路店）</t>
+          <t>沈大成</t>
         </is>
       </c>
     </row>
@@ -2090,79 +2090,79 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>大壶春（四川中路店）</t>
+          <t>莱莱小笼包（南京东路店）</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/09/2027</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>猪手饭（皮诺丘乡村厨房）</t>
+          <t>大壶春（四川中路店）</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/09/2027</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>新旺茶餐室（迪士尼小镇）</t>
+          <t>老吉士（久光百货店）</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/09/2027</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>酸萝卜鸭腿（漫月出口餐车）</t>
+          <t>老正兴菜馆（福州路店）</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>万福兴（凤凰街店）</t>
+          <t>猪手饭（皮诺丘乡村厨房）</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>哑巴生煎（海市山塘 45 号）</t>
+          <t>新旺茶餐室（迪士尼小镇）</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>秋娟小吃店</t>
+          <t>酸萝卜鸭腿（漫月出口餐车）</t>
         </is>
       </c>
     </row>
@@ -2174,67 +2174,67 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>沈万三 · 江南卤味（山塘街店）</t>
+          <t>万福兴（凤凰街店）</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>老客满蛋</t>
+          <t>哑巴生煎（海市山塘 45 号）</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>大孃孃苏式糖水（双塔市集店）</t>
+          <t>秋娟小吃店</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>江南米造局（双塔市集店）</t>
+          <t>沈万三 · 江南卤味（山塘街店）</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>苏外婆 · 苏帮菜 · 松鼠桂鱼（平江路总店）</t>
+          <t>蟹皇捞 · 江南蟹黄面（观前街店）</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>新梅华 · 非遗苏帮菜（星悦汇店）</t>
+          <t>松鹤楼（山塘店）</t>
         </is>
       </c>
     </row>
@@ -2246,175 +2246,175 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>松鹤楼（苏州中心商场店）</t>
+          <t>老客满蛋</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>鑫震源 · 苏式大虾生煎（大儒巷店）</t>
+          <t>大孃孃苏式糖水（双塔市集店）</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>滋啦啦油煎铺</t>
+          <t>江南米造局（双塔市集店）</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>锦记糕点铺</t>
+          <t>苏外婆 · 苏帮菜 · 松鼠桂鱼（平江路总店）</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>书生羊肉面</t>
+          <t>新梅华 · 非遗苏帮菜（星悦汇店）</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>永平粉团铺</t>
+          <t>松鹤楼（苏州中心商场店）</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>锦岸私房菜</t>
+          <t>蟹挽晴 · 蟹黄面（平江路店）</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>桥里桥烧饼铺</t>
+          <t>鑫震源 · 苏式大虾生煎（大儒巷店）</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>赵府私厨 · 老杭帮菜（河坊街店）</t>
+          <t>滋啦啦油煎铺</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>知味观</t>
+          <t>锦记糕点铺</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>杭州绿豆糕（河坊街）</t>
+          <t>书生羊肉面</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>富春王记烧饼（中山中路店总店）</t>
+          <t>永平粉团铺</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>红帽叔叔包子</t>
+          <t>锦岸私房菜</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>潘老板炸鸡腿</t>
+          <t>裕生餐馆</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>熨斗大姐 葱包烩儿</t>
+          <t>和聚兴餐厅</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>新疆烤包子</t>
+          <t>桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>李喜欢虾滑</t>
+          <t>赵府私厨 · 老杭帮菜（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -2450,41 +2450,185 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>龙井茉莉花豆浆</t>
+          <t>知味观</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>杭州绿豆糕（河坊街）</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>富春王记烧饼（中山中路店总店）</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>红帽叔叔包子</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>潘老板炸鸡腿</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>熨斗大姐 葱包烩儿</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>新疆烤包子</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>李喜欢虾滑</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>龙井茉莉花豆浆</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>王润兴酒楼</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>新白鹿餐厅（龙游路总店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>游埠豆浆（河坊街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>杭州酒家（延安路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>福泉素斋</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>寄畅興 · 百年蟹黄面（湖滨银泰 in77 店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
           <t>03/16/2027</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>

</xml_diff>

<commit_message>
Day 4/5 backups: different picks
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -2222,7 +2222,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>蟹皇捞 · 江南蟹黄面（观前街店）</t>
+          <t>朱鸿兴（观前店）</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>松鹤楼（山塘店）</t>
+          <t>俞长盛 · 非遗苏州菜（山塘街店）</t>
         </is>
       </c>
     </row>
@@ -2318,7 +2318,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>蟹挽晴 · 蟹黄面（平江路店）</t>
+          <t>老盛昌汤包（大儒巷店）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day 3: in-park food
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -1943,7 +1943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B57"/>
+  <dimension ref="A1:B61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2169,48 +2169,48 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>万福兴（凤凰街店）</t>
+          <t>米奇好伙伴美味集市</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>哑巴生煎（海市山塘 45 号）</t>
+          <t>星露台餐厅</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>秋娟小吃店</t>
+          <t>巴波萨烧烤</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>沈万三 · 江南卤味（山塘街店）</t>
+          <t>达菲好友欢庆堂</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>朱鸿兴（观前店）</t>
+          <t>万福兴（凤凰街店）</t>
         </is>
       </c>
     </row>
@@ -2234,55 +2234,55 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>俞长盛 · 非遗苏州菜（山塘街店）</t>
+          <t>哑巴生煎（海市山塘 45 号）</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>老客满蛋</t>
+          <t>秋娟小吃店</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>大孃孃苏式糖水（双塔市集店）</t>
+          <t>沈万三 · 江南卤味（山塘街店）</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>江南米造局（双塔市集店）</t>
+          <t>朱鸿兴（观前店）</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>苏外婆 · 苏帮菜 · 松鼠桂鱼（平江路总店）</t>
+          <t>俞长盛 · 非遗苏州菜（山塘街店）</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>新梅华 · 非遗苏帮菜（星悦汇店）</t>
+          <t>老客满蛋</t>
         </is>
       </c>
     </row>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>松鹤楼（苏州中心商场店）</t>
+          <t>大孃孃苏式糖水（双塔市集店）</t>
         </is>
       </c>
     </row>
@@ -2318,55 +2318,55 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>老盛昌汤包（大儒巷店）</t>
+          <t>江南米造局（双塔市集店）</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>鑫震源 · 苏式大虾生煎（大儒巷店）</t>
+          <t>苏外婆 · 苏帮菜 · 松鼠桂鱼（平江路总店）</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>滋啦啦油煎铺</t>
+          <t>新梅华 · 非遗苏帮菜（星悦汇店）</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>锦记糕点铺</t>
+          <t>松鹤楼（苏州中心商场店）</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>书生羊肉面</t>
+          <t>老盛昌汤包（大儒巷店）</t>
         </is>
       </c>
     </row>
@@ -2378,7 +2378,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>永平粉团铺</t>
+          <t>鑫震源 · 苏式大虾生煎（大儒巷店）</t>
         </is>
       </c>
     </row>
@@ -2390,7 +2390,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>锦岸私房菜</t>
+          <t>滋啦啦油煎铺</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>裕生餐馆</t>
+          <t>锦记糕点铺</t>
         </is>
       </c>
     </row>
@@ -2414,55 +2414,55 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>和聚兴餐厅</t>
+          <t>书生羊肉面</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>桥里桥烧饼铺</t>
+          <t>永平粉团铺</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>赵府私厨 · 老杭帮菜（河坊街店）</t>
+          <t>锦岸私房菜</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>知味观</t>
+          <t>裕生餐馆</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>杭州绿豆糕（河坊街）</t>
+          <t>和聚兴餐厅</t>
         </is>
       </c>
     </row>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>富春王记烧饼（中山中路店总店）</t>
+          <t>桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>红帽叔叔包子</t>
+          <t>赵府私厨 · 老杭帮菜（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2498,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>潘老板炸鸡腿</t>
+          <t>知味观</t>
         </is>
       </c>
     </row>
@@ -2510,7 +2510,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>熨斗大姐 葱包烩儿</t>
+          <t>杭州绿豆糕（河坊街）</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>新疆烤包子</t>
+          <t>富春王记烧饼（中山中路店总店）</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>李喜欢虾滑</t>
+          <t>红帽叔叔包子</t>
         </is>
       </c>
     </row>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>龙井茉莉花豆浆</t>
+          <t>潘老板炸鸡腿</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>王润兴酒楼</t>
+          <t>熨斗大姐 葱包烩儿</t>
         </is>
       </c>
     </row>
@@ -2570,65 +2570,113 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>新白鹿餐厅（龙游路总店）</t>
+          <t>新疆烤包子</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>李喜欢虾滑</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>龙井茉莉花豆浆</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>福泉素斋</t>
+          <t>王润兴酒楼</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>寄畅興 · 百年蟹黄面（湖滨银泰 in77 店）</t>
+          <t>新白鹿餐厅（龙游路总店）</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>游埠豆浆（河坊街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>杭州酒家（延安路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>福泉素斋</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>寄畅興 · 百年蟹黄面（湖滨银泰 in77 店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
           <t>03/16/2027</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>

</xml_diff>

<commit_message>
Food tab: drinks for day 2, 5, 6
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -1943,7 +1943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2133,48 +2133,48 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/09/2027</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>猪手饭（皮诺丘乡村厨房）</t>
+          <t>去茶山（兴业太古汇店）</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/09/2027</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>新旺茶餐室（迪士尼小镇）</t>
+          <t>Charlie Town 红茶（静安嘉里中心南区店）</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/09/2027</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>酸萝卜鸭腿（漫月出口餐车）</t>
+          <t>红楼 HONGLOU Gelato（静安嘉里中心店）</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>03/10/2027</t>
+          <t>03/09/2027</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>米奇好伙伴美味集市</t>
+          <t>阿嬷手作（兴业太古汇店）</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>星露台餐厅</t>
+          <t>猪手饭（皮诺丘乡村厨房）</t>
         </is>
       </c>
     </row>
@@ -2198,7 +2198,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>巴波萨烧烤</t>
+          <t>新旺茶餐室（迪士尼小镇）</t>
         </is>
       </c>
     </row>
@@ -2210,55 +2210,55 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>达菲好友欢庆堂</t>
+          <t>酸萝卜鸭腿（漫月出口餐车）</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>万福兴（凤凰街店）</t>
+          <t>米奇好伙伴美味集市</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>哑巴生煎（海市山塘 45 号）</t>
+          <t>星露台餐厅</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>秋娟小吃店</t>
+          <t>巴波萨烧烤</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>03/11/2027</t>
+          <t>03/10/2027</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>沈万三 · 江南卤味（山塘街店）</t>
+          <t>达菲好友欢庆堂</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>朱鸿兴（观前店）</t>
+          <t>万福兴（凤凰街店）</t>
         </is>
       </c>
     </row>
@@ -2282,55 +2282,55 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>俞长盛 · 非遗苏州菜（山塘街店）</t>
+          <t>哑巴生煎（海市山塘 45 号）</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>老客满蛋</t>
+          <t>秋娟小吃店</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>大孃孃苏式糖水（双塔市集店）</t>
+          <t>沈万三 · 江南卤味（山塘街店）</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>江南米造局（双塔市集店）</t>
+          <t>朱鸿兴（观前店）</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/11/2027</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>苏外婆 · 苏帮菜 · 松鼠桂鱼（平江路总店）</t>
+          <t>俞长盛 · 非遗苏州菜（山塘街店）</t>
         </is>
       </c>
     </row>
@@ -2342,7 +2342,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>新梅华 · 非遗苏帮菜（星悦汇店）</t>
+          <t>老客满蛋</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>松鹤楼（苏州中心商场店）</t>
+          <t>大孃孃苏式糖水（双塔市集店）</t>
         </is>
       </c>
     </row>
@@ -2366,79 +2366,79 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>老盛昌汤包（大儒巷店）</t>
+          <t>江南米造局（双塔市集店）</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>鑫震源 · 苏式大虾生煎（大儒巷店）</t>
+          <t>苏外婆 · 苏帮菜 · 松鼠桂鱼（平江路总店）</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>滋啦啦油煎铺</t>
+          <t>新梅华 · 非遗苏帮菜（星悦汇店）</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>锦记糕点铺</t>
+          <t>松鹤楼（苏州中心商场店）</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>书生羊肉面</t>
+          <t>老盛昌汤包（大儒巷店）</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>永平粉团铺</t>
+          <t>三万昌（平江路 1 店）</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>锦岸私房菜</t>
+          <t>羍咖啡馆（羍市咖啡）</t>
         </is>
       </c>
     </row>
@@ -2450,7 +2450,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>裕生餐馆</t>
+          <t>鑫震源 · 苏式大虾生煎（大儒巷店）</t>
         </is>
       </c>
     </row>
@@ -2462,103 +2462,103 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>和聚兴餐厅</t>
+          <t>滋啦啦油煎铺</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>桥里桥烧饼铺</t>
+          <t>锦记糕点铺</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>赵府私厨 · 老杭帮菜（河坊街店）</t>
+          <t>书生羊肉面</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>知味观</t>
+          <t>永平粉团铺</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>杭州绿豆糕（河坊街）</t>
+          <t>锦岸私房菜</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>富春王记烧饼（中山中路店总店）</t>
+          <t>裕生餐馆</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>红帽叔叔包子</t>
+          <t>和聚兴餐厅</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>潘老板炸鸡腿</t>
+          <t>步步莲花咖啡吧</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>03/14/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>熨斗大姐 葱包烩儿</t>
+          <t>似水年华</t>
         </is>
       </c>
     </row>
@@ -2570,7 +2570,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>新疆烤包子</t>
+          <t>桥里桥烧饼铺</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>李喜欢虾滑</t>
+          <t>赵府私厨 · 老杭帮菜（河坊街店）</t>
         </is>
       </c>
     </row>
@@ -2594,7 +2594,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>龙井茉莉花豆浆</t>
+          <t>知味观</t>
         </is>
       </c>
     </row>
@@ -2606,7 +2606,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>王润兴酒楼</t>
+          <t>杭州绿豆糕（河坊街）</t>
         </is>
       </c>
     </row>
@@ -2618,65 +2618,161 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>新白鹿餐厅（龙游路总店）</t>
+          <t>富春王记烧饼（中山中路店总店）</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>游埠豆浆（河坊街店）</t>
+          <t>红帽叔叔包子</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>杭州酒家（延安路店）</t>
+          <t>潘老板炸鸡腿</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>福泉素斋</t>
+          <t>熨斗大姐 葱包烩儿</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/14/2027</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>寄畅興 · 百年蟹黄面（湖滨银泰 in77 店）</t>
+          <t>新疆烤包子</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>李喜欢虾滑</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>龙井茉莉花豆浆</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>王润兴酒楼</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>03/14/2027</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>新白鹿餐厅（龙游路总店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>游埠豆浆（河坊街店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>杭州酒家（延安路店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>福泉素斋</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>寄畅興 · 百年蟹黄面（湖滨银泰 in77 店）</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
           <t>03/16/2027</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t>泮芳春煎饺 · 米其林餐厅（中山南路店）</t>
         </is>

</xml_diff>